<commit_message>
feat: add animal home economy and first-hero rarity reveal
</commit_message>
<xml_diff>
--- a/PM/feature_progress.xlsx
+++ b/PM/feature_progress.xlsx
@@ -8,6 +8,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Capacity" sheetId="4" r:id="R7f249c308d8a4d5f"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Rules" sheetId="5" r:id="R47976c76984c4371"/>
   </x:sheets>
+  <x:calcPr fullCalcOnLoad="1" forceFullCalc="1"/>
 </x:workbook>
 </file>
 
@@ -1147,6 +1148,192 @@
         <x:v>FigJam unavailable; human portraits NOT_RUNTIME; KDF/TLS/rate-limit/Aliyun authorization pending</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="75" customHeight="1">
+      <x:c r="A24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>F-ZC-HOME-001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>动物家园与每日收益</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Filed producer request + DOCX + CSV</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>docs/HOMESTEAD_DESIGN_v1.0.docx</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>config/tables/home_economy.csv; config/tables/home_buildings.csv</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>最多补领3天；解锁地块立即获得1抽卡券</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>P1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H24" s="32">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="I24" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J24" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Not needed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L24" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M24" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Not needed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O24" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P24" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q24" s="32">
+        <x:f>AVERAGE(H24:P24)</x:f>
+        <x:v>0.9857142857142858</x:v>
+      </x:c>
+      <x:c r="R24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Local runtime validated</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="S24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>codex-primary</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="T24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Authorized Aliyun update; device acceptance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="U24" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Formal Figma diagrams unavailable; server deployment and Android not run</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="75" customHeight="1">
+      <x:c r="A25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>F-ZC-GACHA-NEW-001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>新动物品质揭晓与特写</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Filed producer request + DOCX + code</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>docs/HOMESTEAD_DESIGN_v1.0.docx</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Existing card rarity definitions</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>先出品质；点击或等待2秒后显示对应品质色的英雄特写</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>P1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H25" s="32">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="I25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Not needed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J25" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Not needed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L25" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M25" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Not needed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O25" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P25" s="32">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q25" s="32">
+        <x:f>AVERAGE(H25:P25)</x:f>
+        <x:v>0.9833333333333334</x:v>
+      </x:c>
+      <x:c r="R25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Local runtime validated</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="S25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>codex-primary</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="T25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Android export/device acceptance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="U25" s="32" t="inlineStr">
+        <x:is>
+          <x:t>Formal Figma diagrams unavailable; Android not run</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:U2"/>
@@ -1236,7 +1423,7 @@
     <x:row r="5">
       <x:c r="A5" s="27" t="n">
         <x:f>COUNTA('Nine Dimensions'!$A$18:$A$117)</x:f>
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B5" s="27" t="n">
         <x:v>0</x:v>

</xml_diff>

<commit_message>
fix: deploy home construction and restore castle with ring art and gacha polish
</commit_message>
<xml_diff>
--- a/PM/feature_progress.xlsx
+++ b/PM/feature_progress.xlsx
@@ -1166,7 +1166,7 @@
       </x:c>
       <x:c r="D24" s="32" t="inlineStr">
         <x:is>
-          <x:t>docs/HOMESTEAD_DESIGN_v1.0.docx</x:t>
+          <x:t>docs/HOMESTEAD_DESIGN_v1.1.docx</x:t>
         </x:is>
       </x:c>
       <x:c r="E24" s="32" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </x:c>
       <x:c r="F24" s="32" t="inlineStr">
         <x:is>
-          <x:t>最多补领3天；解锁地块立即获得1抽卡券</x:t>
+          <x:t>无建筑升级；按圈数固定外观；足额点击解锁；最多补领3天；解锁赠1券</x:t>
         </x:is>
       </x:c>
       <x:c r="G24" s="32" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </x:c>
       <x:c r="R24" s="32" t="inlineStr">
         <x:is>
-          <x:t>Local runtime validated</x:t>
+          <x:t>Staging home deployed; local UI validated</x:t>
         </x:is>
       </x:c>
       <x:c r="S24" s="32" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </x:c>
       <x:c r="T24" s="32" t="inlineStr">
         <x:is>
-          <x:t>Authorized Aliyun update; device acceptance</x:t>
+          <x:t>External authenticated end-to-end acceptance; Android device acceptance</x:t>
         </x:is>
       </x:c>
       <x:c r="U24" s="32" t="inlineStr">
         <x:is>
-          <x:t>Formal Figma diagrams unavailable; server deployment and Android not run</x:t>
+          <x:t>No real-account writes; external authenticated probe blocked by policy; Figma pending; Android not run</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1258,7 +1258,7 @@
       </x:c>
       <x:c r="D25" s="32" t="inlineStr">
         <x:is>
-          <x:t>docs/HOMESTEAD_DESIGN_v1.0.docx</x:t>
+          <x:t>docs/HOMESTEAD_DESIGN_v1.1.docx</x:t>
         </x:is>
       </x:c>
       <x:c r="E25" s="32" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </x:c>
       <x:c r="F25" s="32" t="inlineStr">
         <x:is>
-          <x:t>先出品质；点击或等待2秒后显示对应品质色的英雄特写</x:t>
+          <x:t>全品质首次获得演出；柔和惊喜音；抽卡不显示等级和升级信息</x:t>
         </x:is>
       </x:c>
       <x:c r="G25" s="32" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </x:c>
       <x:c r="U25" s="32" t="inlineStr">
         <x:is>
-          <x:t>Formal Figma diagrams unavailable; Android not run</x:t>
+          <x:t>All 4 qualities and 60 heroes verified; owned duplicates do not trigger new-hero reveal; Figma pending; Android not run</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>